<commit_message>
feat: croqui das medidas externas do aeroseparador e do silo
Etapa 2 do croqui (aprovada em 26/10, ver docs/croqui.md).

- Item deduzido "MEDIDAS EXTERNAS" pela 1ª palavra do nome do
  equipamento (AEROSEPARADOR, SILO), na guia nova "Exterior".
- Croqui cilindro + cone com as cotas por letra: vazia = falta, cheia =
  medida, cinza = sem acesso ou não tem. Tocar na letra leva ao campo.
- Campos com "Sem acesso" (só com o campo vazio), "Não tem",
  "≈ Estimado" e o Ø pelo perímetro (trena em volta). "sem acesso" e
  "≈" ficam no próprio texto: banco e backup não mudam.
- Planilha: "Fora do PCM" com "A — Ø do corpo: 1910 mm (perímetro
  6000 mm ÷ π); …".
- Celular com o PCM já importado: reimportar o mesmo arquivo cria o
  item sem perder medida (testado).
- Fixture ganha um aeroseparador fictício (XB-AS-01).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XE8a5bB6RCiaHm99L432o7
</commit_message>
<xml_diff>
--- a/tests/fixtures/pcm-ficticio.xlsx
+++ b/tests/fixtures/pcm-ficticio.xlsx
@@ -2690,7 +2690,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W20"/>
+  <dimension ref="A1:W24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3546,22 +3546,22 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>VALVULA PENDULAR - DESCARGA - XB-VV-04</v>
+        <v>AEROSEPARADOR 01 - XB-AS-01</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>MOTOR</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>20 CV 1750RPM</v>
       </c>
       <c r="D13" t="str">
         <v>1 UNIDADE</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>V</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>L</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -3617,13 +3617,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>UNIDADE HIDRÁULICA XB-UH-01</v>
+        <v/>
       </c>
       <c r="B14" t="str">
-        <v>PISTÃO DA UNID. HIDRÁULICA</v>
+        <v>POLIA DO MOTOR</v>
       </c>
       <c r="C14" t="str">
-        <v>CILINDRO 63X400</v>
+        <v>200 4 GORNES B</v>
       </c>
       <c r="D14" t="str">
         <v>1 UNIDADE</v>
@@ -3691,13 +3691,13 @@
         <v/>
       </c>
       <c r="B15" t="str">
-        <v>TERMOPAR XB-TE-01</v>
+        <v>CORREIA EM V</v>
       </c>
       <c r="C15" t="str">
-        <v>TERMOPAR TIPO K</v>
+        <v>B 60</v>
       </c>
       <c r="D15" t="str">
-        <v>1 UNIDADE</v>
+        <v>4 UNIDADES</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -3759,16 +3759,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>OBSERVAÇÕES</v>
+        <v/>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v>RODA DO AERO</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>ROTOR 12 PÁS RETAS</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>1 UNIDADE</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -3830,7 +3830,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>VERIFICAÇÃO E LIMPEZA DE MOTORES, QUINZENAL, PRIMEIRA E TERCEIRA SEMANA DO MÊS</v>
+        <v>VALVULA PENDULAR - DESCARGA - XB-VV-04</v>
       </c>
       <c r="B17" t="str">
         <v/>
@@ -3839,7 +3839,7 @@
         <v/>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>1 UNIDADE</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -3901,13 +3901,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>UNIDADE HIDRÁULICA XB-UH-01</v>
       </c>
       <c r="B18" t="str">
-        <v>ITEM DEPOIS DO RODAPÉ</v>
+        <v>PISTÃO DA UNID. HIDRÁULICA</v>
       </c>
       <c r="C18" t="str">
-        <v>NÃO PODE SER LIDO</v>
+        <v>CILINDRO 63X400</v>
       </c>
       <c r="D18" t="str">
         <v>1 UNIDADE</v>
@@ -3972,16 +3972,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>RESPONSÁVEL PELA INSPEÇÃO/MANUTENÇÃO</v>
+        <v/>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>TERMOPAR XB-TE-01</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>TERMOPAR TIPO K</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>1 UNIDADE</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -4043,82 +4043,367 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>OBSERVAÇÕES</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>VERIFICAÇÃO E LIMPEZA DE MOTORES, QUINZENAL, PRIMEIRA E TERCEIRA SEMANA DO MÊS</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+      <c r="B22" t="str">
+        <v>ITEM DEPOIS DO RODAPÉ</v>
+      </c>
+      <c r="C22" t="str">
+        <v>NÃO PODE SER LIDO</v>
+      </c>
+      <c r="D22" t="str">
+        <v>1 UNIDADE</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>RESPONSÁVEL PELA INSPEÇÃO/MANUTENÇÃO</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>REVISÃO : 01 DATA: 01/01/2024</v>
       </c>
-      <c r="B20" t="str">
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
-        <v/>
-      </c>
-      <c r="G20" t="str">
-        <v/>
-      </c>
-      <c r="H20" t="str">
-        <v/>
-      </c>
-      <c r="I20" t="str">
-        <v/>
-      </c>
-      <c r="J20" t="str">
-        <v/>
-      </c>
-      <c r="K20" t="str">
-        <v/>
-      </c>
-      <c r="L20" t="str">
-        <v/>
-      </c>
-      <c r="M20" t="str">
-        <v/>
-      </c>
-      <c r="N20" t="str">
-        <v/>
-      </c>
-      <c r="O20" t="str">
-        <v/>
-      </c>
-      <c r="P20" t="str">
-        <v/>
-      </c>
-      <c r="Q20" t="str">
-        <v/>
-      </c>
-      <c r="R20" t="str">
-        <v/>
-      </c>
-      <c r="S20" t="str">
-        <v/>
-      </c>
-      <c r="T20" t="str">
-        <v/>
-      </c>
-      <c r="U20" t="str">
-        <v/>
-      </c>
-      <c r="V20" t="str">
-        <v/>
-      </c>
-      <c r="W20" t="str">
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A8:A12"/>
-    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A18:A19"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: croqui dos outros 7 formatos de equipamento
Etapa 3 do croqui (ver docs/croqui.md): peneira, filtro de mangas,
moinho/britador, exaustor/recirculador, rosca, elevador de canecas e
válvula, detectados pela 1ª palavra do nome do equipamento.

- Desenhos com as cotas por letra, num chunk carregado sob demanda
  (fica no precache; o chunk principal não cresce com eles).
- Campos de opção no croqui (nº de decks, tubo ou calha), com
  "Sem acesso".
- Fixture com um equipamento fictício de cada categoria; o E2E abre
  os 24 desenhos e confere a leitura em 360 px.
- PCM real (só contagens): 39 croquis, 0 de 3.073 células alteradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XE8a5bB6RCiaHm99L432o7
</commit_message>
<xml_diff>
--- a/tests/fixtures/pcm-ficticio.xlsx
+++ b/tests/fixtures/pcm-ficticio.xlsx
@@ -2690,7 +2690,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W24"/>
+  <dimension ref="A1:W30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4043,22 +4043,22 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>OBSERVAÇÕES</v>
+        <v>SILO DE CAL - XB-SL-01</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>MOTOR</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>3 CV 1720RPM</v>
       </c>
       <c r="D20" t="str">
-        <v/>
+        <v>1 UNIDADE</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>V</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>L</v>
       </c>
       <c r="G20" t="str">
         <v/>
@@ -4114,16 +4114,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>VERIFICAÇÃO E LIMPEZA DE MOTORES, QUINZENAL, PRIMEIRA E TERCEIRA SEMANA DO MÊS</v>
+        <v>FILTRO DE MANGAS - XB-FM-01</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>MANGAS</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>MANGA POLIESTER 130X3000</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>96 UNIDADES</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -4188,19 +4188,19 @@
         <v/>
       </c>
       <c r="B22" t="str">
-        <v>ITEM DEPOIS DO RODAPÉ</v>
+        <v>MOTOR</v>
       </c>
       <c r="C22" t="str">
-        <v>NÃO PODE SER LIDO</v>
+        <v>1 CV 1720RPM</v>
       </c>
       <c r="D22" t="str">
         <v>1 UNIDADE</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>V</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>L</v>
       </c>
       <c r="G22" t="str">
         <v/>
@@ -4256,22 +4256,22 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>RESPONSÁVEL PELA INSPEÇÃO/MANUTENÇÃO</v>
+        <v>MOINHO DE MARTELOS - XB-MO-01</v>
       </c>
       <c r="B23" t="str">
-        <v/>
+        <v>MOTOR</v>
       </c>
       <c r="C23" t="str">
-        <v/>
+        <v>50 CV 1780RPM</v>
       </c>
       <c r="D23" t="str">
-        <v/>
+        <v>1 UNIDADE</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>V</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>L</v>
       </c>
       <c r="G23" t="str">
         <v/>
@@ -4327,83 +4327,510 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>EXAUSTOR DO FILTRO - XB-EX-01</v>
+      </c>
+      <c r="B24" t="str">
+        <v>MOTOR</v>
+      </c>
+      <c r="C24" t="str">
+        <v>15 CV 3500RPM</v>
+      </c>
+      <c r="D24" t="str">
+        <v>1 UNIDADE</v>
+      </c>
+      <c r="E24" t="str">
+        <v>V</v>
+      </c>
+      <c r="F24" t="str">
+        <v>L</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>ROSCA TRANSPORTADORA - XB-RT-01</v>
+      </c>
+      <c r="B25" t="str">
+        <v>MOTORREDUTOR</v>
+      </c>
+      <c r="C25" t="str">
+        <v>GD40 1:20 3CV 4P</v>
+      </c>
+      <c r="D25" t="str">
+        <v>1 UNIDADE</v>
+      </c>
+      <c r="E25" t="str">
+        <v>V</v>
+      </c>
+      <c r="F25" t="str">
+        <v>L</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
+      <c r="W25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>OBSERVAÇÕES</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>VERIFICAÇÃO E LIMPEZA DE MOTORES, QUINZENAL, PRIMEIRA E TERCEIRA SEMANA DO MÊS</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v/>
+      </c>
+      <c r="B28" t="str">
+        <v>ITEM DEPOIS DO RODAPÉ</v>
+      </c>
+      <c r="C28" t="str">
+        <v>NÃO PODE SER LIDO</v>
+      </c>
+      <c r="D28" t="str">
+        <v>1 UNIDADE</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+      <c r="V28" t="str">
+        <v/>
+      </c>
+      <c r="W28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>RESPONSÁVEL PELA INSPEÇÃO/MANUTENÇÃO</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v>REVISÃO : 01 DATA: 01/01/2024</v>
       </c>
-      <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v/>
-      </c>
-      <c r="D24" t="str">
-        <v/>
-      </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
-        <v/>
-      </c>
-      <c r="G24" t="str">
-        <v/>
-      </c>
-      <c r="H24" t="str">
-        <v/>
-      </c>
-      <c r="I24" t="str">
-        <v/>
-      </c>
-      <c r="J24" t="str">
-        <v/>
-      </c>
-      <c r="K24" t="str">
-        <v/>
-      </c>
-      <c r="L24" t="str">
-        <v/>
-      </c>
-      <c r="M24" t="str">
-        <v/>
-      </c>
-      <c r="N24" t="str">
-        <v/>
-      </c>
-      <c r="O24" t="str">
-        <v/>
-      </c>
-      <c r="P24" t="str">
-        <v/>
-      </c>
-      <c r="Q24" t="str">
-        <v/>
-      </c>
-      <c r="R24" t="str">
-        <v/>
-      </c>
-      <c r="S24" t="str">
-        <v/>
-      </c>
-      <c r="T24" t="str">
-        <v/>
-      </c>
-      <c r="U24" t="str">
-        <v/>
-      </c>
-      <c r="V24" t="str">
-        <v/>
-      </c>
-      <c r="W24" t="str">
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+      <c r="T30" t="str">
+        <v/>
+      </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+      <c r="V30" t="str">
+        <v/>
+      </c>
+      <c r="W30" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A21:A22"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>